<commit_message>
Add prior-year harvest columns to downloadable hunt tables
</commit_message>
<xml_diff>
--- a/processed_data/hard_data_exports/hunt_tables/2026/2026_BISON_COW.xlsx
+++ b/processed_data/hard_data_exports/hunt_tables/2026/2026_BISON_COW.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026_bison_cow" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026_bison_cow" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026_bison_cow'!$A$3:$J$8</definedName>
@@ -539,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.35" customWidth="1" min="1" max="1"/>
@@ -614,6 +614,26 @@
           <t>Total</t>
         </is>
       </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Harvest Prior Year</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Harvest Success (Prior Year %)</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>Average Harvest Age (Prior Year)</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Average Days Hunted (Prior Year)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -666,6 +686,20 @@
           <t>11</t>
         </is>
       </c>
+      <c r="K4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>78.6</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -718,6 +752,20 @@
           <t>11</t>
         </is>
       </c>
+      <c r="K5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>93.1</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -770,6 +818,20 @@
           <t>8</t>
         </is>
       </c>
+      <c r="K6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -820,6 +882,20 @@
       <c r="J7" s="8" t="inlineStr">
         <is>
           <t>15</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>66.7</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>4.3</t>
         </is>
       </c>
     </row>

</xml_diff>